<commit_message>
Update SpaceX valuation model
</commit_message>
<xml_diff>
--- a/07_Model/SpaceX Valuation Model v26.06.11 (Pre-IPO).xlsx
+++ b/07_Model/SpaceX Valuation Model v26.06.11 (Pre-IPO).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\Personal Finances\4-Trades &amp; Investments\Valuation Models\$SPCX - Space Exploration Technologies Corp\07_Model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67B520D8-C626-436F-A73D-F3577D97866F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51DC140B-610F-4341-A95D-8F6BFD033224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="877" xr2:uid="{80111FE1-D860-9C46-9D05-D269D00C2A2F}"/>
   </bookViews>
@@ -19607,7 +19607,7 @@
     <t>Comp Data Status</t>
   </si>
   <si>
-    <t>Rifat Tahmid</t>
+    <t>Property of Rifat Tahmid</t>
   </si>
 </sst>
 </file>
@@ -21237,35 +21237,35 @@
     <xf numFmtId="0" fontId="76" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="78" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="53" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="67" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="53" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="66" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="68" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="17" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="66" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="66" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="54" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="67" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="78" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -23512,33 +23512,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="30" customHeight="1">
-      <c r="A1" s="345" t="s">
+      <c r="A1" s="343" t="s">
         <v>763</v>
       </c>
-      <c r="B1" s="346"/>
-      <c r="C1" s="346"/>
-      <c r="D1" s="346"/>
-      <c r="E1" s="346"/>
-      <c r="F1" s="346"/>
-      <c r="G1" s="346"/>
-      <c r="H1" s="346"/>
-      <c r="I1" s="346"/>
-      <c r="J1" s="346"/>
+      <c r="B1" s="344"/>
+      <c r="C1" s="344"/>
+      <c r="D1" s="344"/>
+      <c r="E1" s="344"/>
+      <c r="F1" s="344"/>
+      <c r="G1" s="344"/>
+      <c r="H1" s="344"/>
+      <c r="I1" s="344"/>
+      <c r="J1" s="344"/>
     </row>
     <row r="2" spans="1:10">
-      <c r="A2" s="347" t="str">
+      <c r="A2" s="345" t="str">
         <f ca="1">"Prepared: "&amp;TEXT(TODAY(),"d-mmm-yyyy")&amp;"  |  Source: SpaceX S-1 (Filed 20-May-2026) "</f>
         <v xml:space="preserve">Prepared: 11-Jun-2026  |  Source: SpaceX S-1 (Filed 20-May-2026) </v>
       </c>
-      <c r="B2" s="348"/>
-      <c r="C2" s="348"/>
-      <c r="D2" s="348"/>
-      <c r="E2" s="348"/>
-      <c r="F2" s="348"/>
-      <c r="G2" s="348"/>
-      <c r="H2" s="348"/>
-      <c r="I2" s="348"/>
-      <c r="J2" s="348"/>
+      <c r="B2" s="346"/>
+      <c r="C2" s="346"/>
+      <c r="D2" s="346"/>
+      <c r="E2" s="346"/>
+      <c r="F2" s="346"/>
+      <c r="G2" s="346"/>
+      <c r="H2" s="346"/>
+      <c r="I2" s="346"/>
+      <c r="J2" s="346"/>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="252"/>
@@ -24641,26 +24641,26 @@
       <c r="F69" s="252"/>
     </row>
     <row r="70" spans="1:10">
-      <c r="A70" s="340" t="s">
+      <c r="A70" s="349" t="s">
         <v>741</v>
       </c>
-      <c r="B70" s="340"/>
-      <c r="C70" s="340" t="s">
+      <c r="B70" s="349"/>
+      <c r="C70" s="349" t="s">
         <v>742</v>
       </c>
-      <c r="D70" s="340"/>
-      <c r="E70" s="340"/>
-      <c r="F70" s="340"/>
-      <c r="G70" s="340"/>
-      <c r="H70" s="340"/>
-      <c r="I70" s="340"/>
-      <c r="J70" s="340"/>
+      <c r="D70" s="349"/>
+      <c r="E70" s="349"/>
+      <c r="F70" s="349"/>
+      <c r="G70" s="349"/>
+      <c r="H70" s="349"/>
+      <c r="I70" s="349"/>
+      <c r="J70" s="349"/>
     </row>
     <row r="71" spans="1:10" ht="14.4" customHeight="1">
-      <c r="A71" s="344" t="s">
+      <c r="A71" s="347" t="s">
         <v>743</v>
       </c>
-      <c r="B71" s="344"/>
+      <c r="B71" s="347"/>
       <c r="C71" s="341" t="s">
         <v>744</v>
       </c>
@@ -24673,10 +24673,10 @@
       <c r="J71" s="341"/>
     </row>
     <row r="72" spans="1:10" ht="14.4" customHeight="1">
-      <c r="A72" s="344" t="s">
+      <c r="A72" s="347" t="s">
         <v>745</v>
       </c>
-      <c r="B72" s="344"/>
+      <c r="B72" s="347"/>
       <c r="C72" s="341" t="s">
         <v>746</v>
       </c>
@@ -24689,10 +24689,10 @@
       <c r="J72" s="341"/>
     </row>
     <row r="73" spans="1:10" ht="14.4" customHeight="1">
-      <c r="A73" s="344" t="s">
+      <c r="A73" s="347" t="s">
         <v>747</v>
       </c>
-      <c r="B73" s="344"/>
+      <c r="B73" s="347"/>
       <c r="C73" s="341" t="s">
         <v>748</v>
       </c>
@@ -24705,10 +24705,10 @@
       <c r="J73" s="341"/>
     </row>
     <row r="74" spans="1:10" ht="14.4" customHeight="1">
-      <c r="A74" s="344" t="s">
+      <c r="A74" s="347" t="s">
         <v>749</v>
       </c>
-      <c r="B74" s="344"/>
+      <c r="B74" s="347"/>
       <c r="C74" s="341" t="s">
         <v>750</v>
       </c>
@@ -24721,10 +24721,10 @@
       <c r="J74" s="341"/>
     </row>
     <row r="75" spans="1:10" ht="14.4" customHeight="1">
-      <c r="A75" s="344" t="s">
+      <c r="A75" s="347" t="s">
         <v>751</v>
       </c>
-      <c r="B75" s="344"/>
+      <c r="B75" s="347"/>
       <c r="C75" s="341" t="s">
         <v>752</v>
       </c>
@@ -24737,10 +24737,10 @@
       <c r="J75" s="341"/>
     </row>
     <row r="76" spans="1:10" ht="14.4" customHeight="1">
-      <c r="A76" s="344" t="s">
+      <c r="A76" s="347" t="s">
         <v>57</v>
       </c>
-      <c r="B76" s="344"/>
+      <c r="B76" s="347"/>
       <c r="C76" s="341" t="s">
         <v>753</v>
       </c>
@@ -24753,10 +24753,10 @@
       <c r="J76" s="341"/>
     </row>
     <row r="77" spans="1:10" ht="14.4" customHeight="1">
-      <c r="A77" s="344" t="s">
+      <c r="A77" s="347" t="s">
         <v>754</v>
       </c>
-      <c r="B77" s="344"/>
+      <c r="B77" s="347"/>
       <c r="C77" s="341" t="s">
         <v>755</v>
       </c>
@@ -24769,10 +24769,10 @@
       <c r="J77" s="341"/>
     </row>
     <row r="78" spans="1:10" ht="14.4" customHeight="1">
-      <c r="A78" s="344" t="s">
+      <c r="A78" s="347" t="s">
         <v>756</v>
       </c>
-      <c r="B78" s="344"/>
+      <c r="B78" s="347"/>
       <c r="C78" s="341" t="s">
         <v>757</v>
       </c>
@@ -24785,10 +24785,10 @@
       <c r="J78" s="341"/>
     </row>
     <row r="79" spans="1:10" ht="14.4" customHeight="1">
-      <c r="A79" s="344" t="s">
+      <c r="A79" s="347" t="s">
         <v>758</v>
       </c>
-      <c r="B79" s="344"/>
+      <c r="B79" s="347"/>
       <c r="C79" s="341" t="s">
         <v>759</v>
       </c>
@@ -24801,43 +24801,63 @@
       <c r="J79" s="341"/>
     </row>
     <row r="80" spans="1:10" ht="14.4" customHeight="1">
-      <c r="A80" s="349" t="s">
+      <c r="A80" s="348" t="s">
         <v>760</v>
       </c>
-      <c r="B80" s="349"/>
-      <c r="C80" s="343" t="s">
+      <c r="B80" s="348"/>
+      <c r="C80" s="342" t="s">
         <v>761</v>
       </c>
-      <c r="D80" s="343"/>
-      <c r="E80" s="343"/>
-      <c r="F80" s="343"/>
-      <c r="G80" s="343"/>
-      <c r="H80" s="343"/>
-      <c r="I80" s="343"/>
-      <c r="J80" s="343"/>
+      <c r="D80" s="342"/>
+      <c r="E80" s="342"/>
+      <c r="F80" s="342"/>
+      <c r="G80" s="342"/>
+      <c r="H80" s="342"/>
+      <c r="I80" s="342"/>
+      <c r="J80" s="342"/>
     </row>
     <row r="81" spans="1:10" ht="14.4" customHeight="1"/>
     <row r="82" spans="1:10" ht="21.6" customHeight="1">
-      <c r="A82" s="342" t="s">
+      <c r="A82" s="350" t="s">
         <v>762</v>
       </c>
-      <c r="B82" s="342"/>
-      <c r="C82" s="342"/>
-      <c r="D82" s="342"/>
-      <c r="E82" s="342"/>
-      <c r="F82" s="342"/>
-      <c r="G82" s="342"/>
-      <c r="H82" s="342"/>
-      <c r="I82" s="342"/>
-      <c r="J82" s="342"/>
+      <c r="B82" s="350"/>
+      <c r="C82" s="350"/>
+      <c r="D82" s="350"/>
+      <c r="E82" s="350"/>
+      <c r="F82" s="350"/>
+      <c r="G82" s="350"/>
+      <c r="H82" s="350"/>
+      <c r="I82" s="350"/>
+      <c r="J82" s="350"/>
     </row>
     <row r="100" spans="1:1">
-      <c r="A100" s="356" t="s">
+      <c r="A100" s="340" t="s">
         <v>791</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="36">
+    <mergeCell ref="A82:J82"/>
+    <mergeCell ref="G70:J70"/>
+    <mergeCell ref="G71:J71"/>
+    <mergeCell ref="G72:J72"/>
+    <mergeCell ref="G73:J73"/>
+    <mergeCell ref="G74:J74"/>
+    <mergeCell ref="G75:J75"/>
+    <mergeCell ref="G76:J76"/>
+    <mergeCell ref="C80:F80"/>
+    <mergeCell ref="A70:B70"/>
+    <mergeCell ref="A71:B71"/>
+    <mergeCell ref="A72:B72"/>
+    <mergeCell ref="A74:B74"/>
+    <mergeCell ref="A75:B75"/>
+    <mergeCell ref="A76:B76"/>
+    <mergeCell ref="G77:J77"/>
+    <mergeCell ref="C70:F70"/>
+    <mergeCell ref="C71:F71"/>
+    <mergeCell ref="C72:F72"/>
+    <mergeCell ref="C73:F73"/>
     <mergeCell ref="G78:J78"/>
     <mergeCell ref="G79:J79"/>
     <mergeCell ref="G80:J80"/>
@@ -24854,26 +24874,6 @@
     <mergeCell ref="C78:F78"/>
     <mergeCell ref="C79:F79"/>
     <mergeCell ref="A73:B73"/>
-    <mergeCell ref="A74:B74"/>
-    <mergeCell ref="A75:B75"/>
-    <mergeCell ref="A76:B76"/>
-    <mergeCell ref="G77:J77"/>
-    <mergeCell ref="C70:F70"/>
-    <mergeCell ref="C71:F71"/>
-    <mergeCell ref="C72:F72"/>
-    <mergeCell ref="C73:F73"/>
-    <mergeCell ref="A82:J82"/>
-    <mergeCell ref="G70:J70"/>
-    <mergeCell ref="G71:J71"/>
-    <mergeCell ref="G72:J72"/>
-    <mergeCell ref="G73:J73"/>
-    <mergeCell ref="G74:J74"/>
-    <mergeCell ref="G75:J75"/>
-    <mergeCell ref="G76:J76"/>
-    <mergeCell ref="C80:F80"/>
-    <mergeCell ref="A70:B70"/>
-    <mergeCell ref="A71:B71"/>
-    <mergeCell ref="A72:B72"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -34486,7 +34486,7 @@
       </c>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="350" t="s">
+      <c r="A4" s="351" t="s">
         <v>390</v>
       </c>
       <c r="B4" s="352"/>
@@ -34787,16 +34787,16 @@
       <c r="G16" s="54"/>
     </row>
     <row r="18" spans="1:8">
-      <c r="A18" s="355" t="s">
+      <c r="A18" s="356" t="s">
         <v>392</v>
       </c>
-      <c r="B18" s="355"/>
-      <c r="C18" s="355"/>
-      <c r="D18" s="355"/>
-      <c r="E18" s="355"/>
-      <c r="F18" s="355"/>
-      <c r="G18" s="355"/>
-      <c r="H18" s="355"/>
+      <c r="B18" s="356"/>
+      <c r="C18" s="356"/>
+      <c r="D18" s="356"/>
+      <c r="E18" s="356"/>
+      <c r="F18" s="356"/>
+      <c r="G18" s="356"/>
+      <c r="H18" s="356"/>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="6" t="s">
@@ -34939,16 +34939,16 @@
       </c>
     </row>
     <row r="26" spans="1:8">
-      <c r="A26" s="355" t="s">
+      <c r="A26" s="356" t="s">
         <v>397</v>
       </c>
-      <c r="B26" s="355"/>
-      <c r="C26" s="355"/>
-      <c r="D26" s="355"/>
-      <c r="E26" s="355"/>
-      <c r="F26" s="355"/>
-      <c r="G26" s="355"/>
-      <c r="H26" s="355"/>
+      <c r="B26" s="356"/>
+      <c r="C26" s="356"/>
+      <c r="D26" s="356"/>
+      <c r="E26" s="356"/>
+      <c r="F26" s="356"/>
+      <c r="G26" s="356"/>
+      <c r="H26" s="356"/>
     </row>
     <row r="27" spans="1:8">
       <c r="A27" s="6" t="s">
@@ -35159,16 +35159,16 @@
       <c r="H36" s="54"/>
     </row>
     <row r="38" spans="1:8">
-      <c r="A38" s="355" t="s">
+      <c r="A38" s="356" t="s">
         <v>402</v>
       </c>
-      <c r="B38" s="355"/>
-      <c r="C38" s="355"/>
-      <c r="D38" s="355"/>
-      <c r="E38" s="355"/>
-      <c r="F38" s="355"/>
-      <c r="G38" s="355"/>
-      <c r="H38" s="355"/>
+      <c r="B38" s="356"/>
+      <c r="C38" s="356"/>
+      <c r="D38" s="356"/>
+      <c r="E38" s="356"/>
+      <c r="F38" s="356"/>
+      <c r="G38" s="356"/>
+      <c r="H38" s="356"/>
     </row>
     <row r="39" spans="1:8">
       <c r="A39" s="6" t="s">
@@ -37495,46 +37495,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="30" customHeight="1">
-      <c r="A1" s="345" t="s">
+      <c r="A1" s="343" t="s">
         <v>764</v>
       </c>
-      <c r="B1" s="346"/>
-      <c r="C1" s="346"/>
-      <c r="D1" s="346"/>
-      <c r="E1" s="346"/>
-      <c r="F1" s="346"/>
-      <c r="G1" s="346"/>
-      <c r="H1" s="346"/>
-      <c r="I1" s="346"/>
-      <c r="J1" s="346"/>
+      <c r="B1" s="344"/>
+      <c r="C1" s="344"/>
+      <c r="D1" s="344"/>
+      <c r="E1" s="344"/>
+      <c r="F1" s="344"/>
+      <c r="G1" s="344"/>
+      <c r="H1" s="344"/>
+      <c r="I1" s="344"/>
+      <c r="J1" s="344"/>
     </row>
     <row r="2" spans="1:10">
-      <c r="A2" s="347" t="s">
+      <c r="A2" s="345" t="s">
         <v>193</v>
       </c>
-      <c r="B2" s="348"/>
-      <c r="C2" s="348"/>
-      <c r="D2" s="348"/>
-      <c r="E2" s="348"/>
-      <c r="F2" s="348"/>
-      <c r="G2" s="348"/>
-      <c r="H2" s="348"/>
-      <c r="I2" s="348"/>
-      <c r="J2" s="348"/>
+      <c r="B2" s="346"/>
+      <c r="C2" s="346"/>
+      <c r="D2" s="346"/>
+      <c r="E2" s="346"/>
+      <c r="F2" s="346"/>
+      <c r="G2" s="346"/>
+      <c r="H2" s="346"/>
+      <c r="I2" s="346"/>
+      <c r="J2" s="346"/>
     </row>
     <row r="4" spans="1:10" ht="15" thickBot="1">
-      <c r="A4" s="350" t="s">
+      <c r="A4" s="351" t="s">
         <v>194</v>
       </c>
-      <c r="B4" s="346"/>
-      <c r="C4" s="346"/>
-      <c r="D4" s="346"/>
-      <c r="E4" s="346"/>
-      <c r="F4" s="346"/>
-      <c r="G4" s="346"/>
-      <c r="H4" s="346"/>
-      <c r="I4" s="346"/>
-      <c r="J4" s="346"/>
+      <c r="B4" s="344"/>
+      <c r="C4" s="344"/>
+      <c r="D4" s="344"/>
+      <c r="E4" s="344"/>
+      <c r="F4" s="344"/>
+      <c r="G4" s="344"/>
+      <c r="H4" s="344"/>
+      <c r="I4" s="344"/>
+      <c r="J4" s="344"/>
     </row>
     <row r="5" spans="1:10" ht="15" thickBot="1">
       <c r="A5" s="1" t="s">
@@ -37543,7 +37543,7 @@
       <c r="B5" s="32">
         <v>135</v>
       </c>
-      <c r="C5" s="351" t="s">
+      <c r="C5" s="355" t="s">
         <v>196</v>
       </c>
       <c r="D5" s="352"/>
@@ -37555,18 +37555,18 @@
       <c r="J5" s="352"/>
     </row>
     <row r="7" spans="1:10">
-      <c r="A7" s="350" t="s">
+      <c r="A7" s="351" t="s">
         <v>197</v>
       </c>
-      <c r="B7" s="346"/>
-      <c r="C7" s="346"/>
-      <c r="D7" s="346"/>
-      <c r="E7" s="346"/>
-      <c r="F7" s="346"/>
-      <c r="G7" s="346"/>
-      <c r="H7" s="346"/>
-      <c r="I7" s="346"/>
-      <c r="J7" s="346"/>
+      <c r="B7" s="344"/>
+      <c r="C7" s="344"/>
+      <c r="D7" s="344"/>
+      <c r="E7" s="344"/>
+      <c r="F7" s="344"/>
+      <c r="G7" s="344"/>
+      <c r="H7" s="344"/>
+      <c r="I7" s="344"/>
+      <c r="J7" s="344"/>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="6"/>
@@ -37788,18 +37788,18 @@
       <c r="J18" s="145"/>
     </row>
     <row r="20" spans="1:10">
-      <c r="A20" s="350" t="s">
+      <c r="A20" s="351" t="s">
         <v>243</v>
       </c>
-      <c r="B20" s="346"/>
-      <c r="C20" s="346"/>
-      <c r="D20" s="346"/>
-      <c r="E20" s="346"/>
-      <c r="F20" s="346"/>
-      <c r="G20" s="346"/>
-      <c r="H20" s="346"/>
-      <c r="I20" s="346"/>
-      <c r="J20" s="346"/>
+      <c r="B20" s="344"/>
+      <c r="C20" s="344"/>
+      <c r="D20" s="344"/>
+      <c r="E20" s="344"/>
+      <c r="F20" s="344"/>
+      <c r="G20" s="344"/>
+      <c r="H20" s="344"/>
+      <c r="I20" s="344"/>
+      <c r="J20" s="344"/>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="6"/>
@@ -37877,18 +37877,18 @@
       <c r="J24" s="150"/>
     </row>
     <row r="26" spans="1:10">
-      <c r="A26" s="350" t="s">
+      <c r="A26" s="351" t="s">
         <v>211</v>
       </c>
-      <c r="B26" s="346"/>
-      <c r="C26" s="346"/>
-      <c r="D26" s="346"/>
-      <c r="E26" s="346"/>
-      <c r="F26" s="346"/>
-      <c r="G26" s="346"/>
-      <c r="H26" s="346"/>
-      <c r="I26" s="346"/>
-      <c r="J26" s="346"/>
+      <c r="B26" s="344"/>
+      <c r="C26" s="344"/>
+      <c r="D26" s="344"/>
+      <c r="E26" s="344"/>
+      <c r="F26" s="344"/>
+      <c r="G26" s="344"/>
+      <c r="H26" s="344"/>
+      <c r="I26" s="344"/>
+      <c r="J26" s="344"/>
     </row>
     <row r="27" spans="1:10">
       <c r="A27" s="6" t="s">
@@ -37987,18 +37987,18 @@
       <c r="J31" s="352"/>
     </row>
     <row r="33" spans="1:10">
-      <c r="A33" s="350" t="s">
+      <c r="A33" s="351" t="s">
         <v>232</v>
       </c>
-      <c r="B33" s="346"/>
-      <c r="C33" s="346"/>
-      <c r="D33" s="346"/>
-      <c r="E33" s="346"/>
-      <c r="F33" s="346"/>
-      <c r="G33" s="346"/>
-      <c r="H33" s="346"/>
-      <c r="I33" s="346"/>
-      <c r="J33" s="346"/>
+      <c r="B33" s="344"/>
+      <c r="C33" s="344"/>
+      <c r="D33" s="344"/>
+      <c r="E33" s="344"/>
+      <c r="F33" s="344"/>
+      <c r="G33" s="344"/>
+      <c r="H33" s="344"/>
+      <c r="I33" s="344"/>
+      <c r="J33" s="344"/>
     </row>
     <row r="34" spans="1:10">
       <c r="A34" s="6" t="s">
@@ -38081,18 +38081,18 @@
       <c r="J37" s="150"/>
     </row>
     <row r="39" spans="1:10">
-      <c r="A39" s="350" t="s">
+      <c r="A39" s="351" t="s">
         <v>425</v>
       </c>
-      <c r="B39" s="346"/>
-      <c r="C39" s="346"/>
-      <c r="D39" s="346"/>
-      <c r="E39" s="346"/>
-      <c r="F39" s="346"/>
-      <c r="G39" s="346"/>
-      <c r="H39" s="346"/>
-      <c r="I39" s="346"/>
-      <c r="J39" s="346"/>
+      <c r="B39" s="344"/>
+      <c r="C39" s="344"/>
+      <c r="D39" s="344"/>
+      <c r="E39" s="344"/>
+      <c r="F39" s="344"/>
+      <c r="G39" s="344"/>
+      <c r="H39" s="344"/>
+      <c r="I39" s="344"/>
+      <c r="J39" s="344"/>
     </row>
     <row r="40" spans="1:10">
       <c r="A40" s="6" t="s">
@@ -38254,18 +38254,18 @@
       </c>
     </row>
     <row r="48" spans="1:10">
-      <c r="A48" s="350" t="s">
+      <c r="A48" s="351" t="s">
         <v>219</v>
       </c>
-      <c r="B48" s="346"/>
-      <c r="C48" s="346"/>
-      <c r="D48" s="346"/>
-      <c r="E48" s="346"/>
-      <c r="F48" s="346"/>
-      <c r="G48" s="346"/>
-      <c r="H48" s="346"/>
-      <c r="I48" s="346"/>
-      <c r="J48" s="346"/>
+      <c r="B48" s="344"/>
+      <c r="C48" s="344"/>
+      <c r="D48" s="344"/>
+      <c r="E48" s="344"/>
+      <c r="F48" s="344"/>
+      <c r="G48" s="344"/>
+      <c r="H48" s="344"/>
+      <c r="I48" s="344"/>
+      <c r="J48" s="344"/>
     </row>
     <row r="49" spans="1:10">
       <c r="A49" s="6" t="s">
@@ -38456,7 +38456,7 @@
       </c>
     </row>
     <row r="62" spans="1:10">
-      <c r="A62" s="350" t="s">
+      <c r="A62" s="351" t="s">
         <v>311</v>
       </c>
       <c r="B62" s="352"/>
@@ -38610,6 +38610,12 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A20:J20"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A4:J4"/>
+    <mergeCell ref="C5:J5"/>
+    <mergeCell ref="A7:J7"/>
     <mergeCell ref="A62:J62"/>
     <mergeCell ref="A26:J26"/>
     <mergeCell ref="A31:J31"/>
@@ -38617,12 +38623,6 @@
     <mergeCell ref="A39:J39"/>
     <mergeCell ref="A48:J48"/>
     <mergeCell ref="B34:D34"/>
-    <mergeCell ref="A20:J20"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A4:J4"/>
-    <mergeCell ref="C5:J5"/>
-    <mergeCell ref="A7:J7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -39424,15 +39424,15 @@
       </c>
     </row>
     <row r="48" spans="1:7">
-      <c r="A48" s="350" t="s">
+      <c r="A48" s="351" t="s">
         <v>423</v>
       </c>
-      <c r="B48" s="350"/>
-      <c r="C48" s="350"/>
-      <c r="D48" s="350"/>
-      <c r="E48" s="350"/>
-      <c r="F48" s="350"/>
-      <c r="G48" s="350"/>
+      <c r="B48" s="351"/>
+      <c r="C48" s="351"/>
+      <c r="D48" s="351"/>
+      <c r="E48" s="351"/>
+      <c r="F48" s="351"/>
+      <c r="G48" s="351"/>
     </row>
     <row r="50" spans="1:7">
       <c r="A50" s="22" t="s">
@@ -45105,32 +45105,32 @@
       </c>
     </row>
     <row r="124" spans="1:24">
-      <c r="A124" s="350" t="s">
+      <c r="A124" s="351" t="s">
         <v>265</v>
       </c>
-      <c r="B124" s="350"/>
-      <c r="C124" s="350"/>
-      <c r="D124" s="350"/>
-      <c r="E124" s="350"/>
-      <c r="F124" s="350"/>
-      <c r="G124" s="350"/>
-      <c r="H124" s="350"/>
-      <c r="I124" s="350"/>
-      <c r="J124" s="350"/>
-      <c r="K124" s="350"/>
-      <c r="L124" s="350"/>
-      <c r="M124" s="350"/>
-      <c r="N124" s="350"/>
-      <c r="O124" s="350"/>
-      <c r="P124" s="350"/>
-      <c r="Q124" s="350"/>
-      <c r="R124" s="350"/>
-      <c r="S124" s="350"/>
-      <c r="T124" s="350"/>
-      <c r="U124" s="350"/>
-      <c r="V124" s="350"/>
-      <c r="W124" s="350"/>
-      <c r="X124" s="350"/>
+      <c r="B124" s="351"/>
+      <c r="C124" s="351"/>
+      <c r="D124" s="351"/>
+      <c r="E124" s="351"/>
+      <c r="F124" s="351"/>
+      <c r="G124" s="351"/>
+      <c r="H124" s="351"/>
+      <c r="I124" s="351"/>
+      <c r="J124" s="351"/>
+      <c r="K124" s="351"/>
+      <c r="L124" s="351"/>
+      <c r="M124" s="351"/>
+      <c r="N124" s="351"/>
+      <c r="O124" s="351"/>
+      <c r="P124" s="351"/>
+      <c r="Q124" s="351"/>
+      <c r="R124" s="351"/>
+      <c r="S124" s="351"/>
+      <c r="T124" s="351"/>
+      <c r="U124" s="351"/>
+      <c r="V124" s="351"/>
+      <c r="W124" s="351"/>
+      <c r="X124" s="351"/>
     </row>
     <row r="125" spans="1:24">
       <c r="A125" s="6" t="s">
@@ -51193,32 +51193,32 @@
       </c>
     </row>
     <row r="124" spans="1:24">
-      <c r="A124" s="350" t="s">
+      <c r="A124" s="351" t="s">
         <v>285</v>
       </c>
-      <c r="B124" s="350"/>
-      <c r="C124" s="350"/>
-      <c r="D124" s="350"/>
-      <c r="E124" s="350"/>
-      <c r="F124" s="350"/>
-      <c r="G124" s="350"/>
-      <c r="H124" s="350"/>
-      <c r="I124" s="350"/>
-      <c r="J124" s="350"/>
-      <c r="K124" s="350"/>
-      <c r="L124" s="350"/>
-      <c r="M124" s="350"/>
-      <c r="N124" s="350"/>
-      <c r="O124" s="350"/>
-      <c r="P124" s="350"/>
-      <c r="Q124" s="350"/>
-      <c r="R124" s="350"/>
-      <c r="S124" s="350"/>
-      <c r="T124" s="350"/>
-      <c r="U124" s="350"/>
-      <c r="V124" s="350"/>
-      <c r="W124" s="350"/>
-      <c r="X124" s="350"/>
+      <c r="B124" s="351"/>
+      <c r="C124" s="351"/>
+      <c r="D124" s="351"/>
+      <c r="E124" s="351"/>
+      <c r="F124" s="351"/>
+      <c r="G124" s="351"/>
+      <c r="H124" s="351"/>
+      <c r="I124" s="351"/>
+      <c r="J124" s="351"/>
+      <c r="K124" s="351"/>
+      <c r="L124" s="351"/>
+      <c r="M124" s="351"/>
+      <c r="N124" s="351"/>
+      <c r="O124" s="351"/>
+      <c r="P124" s="351"/>
+      <c r="Q124" s="351"/>
+      <c r="R124" s="351"/>
+      <c r="S124" s="351"/>
+      <c r="T124" s="351"/>
+      <c r="U124" s="351"/>
+      <c r="V124" s="351"/>
+      <c r="W124" s="351"/>
+      <c r="X124" s="351"/>
     </row>
     <row r="125" spans="1:24">
       <c r="A125" s="6" t="s">
@@ -57013,32 +57013,32 @@
       </c>
     </row>
     <row r="124" spans="1:24">
-      <c r="A124" s="350" t="s">
+      <c r="A124" s="351" t="s">
         <v>277</v>
       </c>
-      <c r="B124" s="350"/>
-      <c r="C124" s="350"/>
-      <c r="D124" s="350"/>
-      <c r="E124" s="350"/>
-      <c r="F124" s="350"/>
-      <c r="G124" s="350"/>
-      <c r="H124" s="350"/>
-      <c r="I124" s="350"/>
-      <c r="J124" s="350"/>
-      <c r="K124" s="350"/>
-      <c r="L124" s="350"/>
-      <c r="M124" s="350"/>
-      <c r="N124" s="350"/>
-      <c r="O124" s="350"/>
-      <c r="P124" s="350"/>
-      <c r="Q124" s="350"/>
-      <c r="R124" s="350"/>
-      <c r="S124" s="350"/>
-      <c r="T124" s="350"/>
-      <c r="U124" s="350"/>
-      <c r="V124" s="350"/>
-      <c r="W124" s="350"/>
-      <c r="X124" s="350"/>
+      <c r="B124" s="351"/>
+      <c r="C124" s="351"/>
+      <c r="D124" s="351"/>
+      <c r="E124" s="351"/>
+      <c r="F124" s="351"/>
+      <c r="G124" s="351"/>
+      <c r="H124" s="351"/>
+      <c r="I124" s="351"/>
+      <c r="J124" s="351"/>
+      <c r="K124" s="351"/>
+      <c r="L124" s="351"/>
+      <c r="M124" s="351"/>
+      <c r="N124" s="351"/>
+      <c r="O124" s="351"/>
+      <c r="P124" s="351"/>
+      <c r="Q124" s="351"/>
+      <c r="R124" s="351"/>
+      <c r="S124" s="351"/>
+      <c r="T124" s="351"/>
+      <c r="U124" s="351"/>
+      <c r="V124" s="351"/>
+      <c r="W124" s="351"/>
+      <c r="X124" s="351"/>
     </row>
     <row r="125" spans="1:24">
       <c r="A125" s="6" t="s">
@@ -58694,7 +58694,7 @@
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="350" t="s">
+      <c r="A4" s="351" t="s">
         <v>318</v>
       </c>
       <c r="B4" s="352"/>
@@ -58767,7 +58767,7 @@
       </c>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="350" t="s">
+      <c r="A13" s="351" t="s">
         <v>326</v>
       </c>
       <c r="B13" s="352"/>
@@ -58839,7 +58839,7 @@
       </c>
     </row>
     <row r="22" spans="1:6">
-      <c r="A22" s="350" t="s">
+      <c r="A22" s="351" t="s">
         <v>332</v>
       </c>
       <c r="B22" s="352"/>
@@ -58965,7 +58965,7 @@
       </c>
     </row>
     <row r="31" spans="1:6">
-      <c r="A31" s="350" t="s">
+      <c r="A31" s="351" t="s">
         <v>348</v>
       </c>
       <c r="B31" s="352"/>
@@ -59031,7 +59031,7 @@
       </c>
     </row>
     <row r="40" spans="1:6">
-      <c r="A40" s="350" t="s">
+      <c r="A40" s="351" t="s">
         <v>356</v>
       </c>
       <c r="B40" s="352"/>

</xml_diff>